<commit_message>
In the Works: Drive links from the review email wired into the not-in-Doom rows
Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0161jaxJZTksz7q1T7aevp9F
</commit_message>
<xml_diff>
--- a/lr-in-the-works.xlsx
+++ b/lr-in-the-works.xlsx
@@ -466,7 +466,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S30"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
@@ -607,7 +607,10 @@
           <t>LNR_It's a trap PHX</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr"/>
+      <c r="G2" s="5">
+        <f>HYPERLINK("https://drive.google.com/file/d/10DLmAVoh6a-NIp56bgTiMX6eNVd7-0pf/view","▶ Watch")</f>
+        <v/>
+      </c>
       <c r="H2" s="5" t="inlineStr"/>
       <c r="I2" s="5" t="inlineStr"/>
       <c r="J2" s="5" t="inlineStr"/>
@@ -670,7 +673,10 @@
           <t>LNR_Before and After Phx</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr"/>
+      <c r="G3" s="5">
+        <f>HYPERLINK("https://drive.google.com/file/d/1F8vzl1oQwXTq6T03499Mgljbd-hadA67/view","▶ Watch")</f>
+        <v/>
+      </c>
       <c r="H3" s="5" t="inlineStr"/>
       <c r="I3" s="5" t="inlineStr"/>
       <c r="J3" s="5" t="inlineStr"/>
@@ -733,7 +739,10 @@
           <t>LNR_Different Story</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr"/>
+      <c r="G4" s="5">
+        <f>HYPERLINK("https://drive.google.com/file/d/1oUmXQcLQ7hMTI6nWMLvsNx0D-1klIxcW/view","▶ Watch")</f>
+        <v/>
+      </c>
       <c r="H4" s="5" t="inlineStr"/>
       <c r="I4" s="5" t="inlineStr"/>
       <c r="J4" s="5" t="inlineStr"/>
@@ -796,7 +805,10 @@
           <t>LNR_Amazing Results PHX</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr"/>
+      <c r="G5" s="5">
+        <f>HYPERLINK("https://drive.google.com/file/d/16VgkoHUmwlJvKWPc5ltY_QxZkoh7UKTr/view","▶ Watch")</f>
+        <v/>
+      </c>
       <c r="H5" s="5" t="inlineStr"/>
       <c r="I5" s="5" t="inlineStr"/>
       <c r="J5" s="5" t="inlineStr"/>
@@ -859,7 +871,10 @@
           <t>LNR_So Many PHX</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr"/>
+      <c r="G6" s="5">
+        <f>HYPERLINK("https://drive.google.com/file/d/1d5wbtEvh8ou594Wr4VFFXIW-pnFPZlbj/view","▶ Watch")</f>
+        <v/>
+      </c>
       <c r="H6" s="5" t="inlineStr"/>
       <c r="I6" s="5" t="inlineStr"/>
       <c r="J6" s="5" t="inlineStr"/>
@@ -1004,7 +1019,10 @@
           <t>LNR_Billion dollar firm PHX</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr"/>
+      <c r="G8" s="5">
+        <f>HYPERLINK("https://drive.google.com/file/d/1SG9l5YdUbAxEEBVrzpLGHqvSW2mKIGDu/view","▶ Watch")</f>
+        <v/>
+      </c>
       <c r="H8" s="5" t="inlineStr"/>
       <c r="I8" s="5" t="inlineStr"/>
       <c r="J8" s="5" t="inlineStr"/>
@@ -1137,7 +1155,10 @@
           <t>LNR_Long Distance PHX</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr"/>
+      <c r="G10" s="5">
+        <f>HYPERLINK("https://drive.google.com/file/d/1b8KBNCZdmXRRqWsBiVHNo_oQ49R77S7A/view","▶ Watch")</f>
+        <v/>
+      </c>
       <c r="H10" s="5" t="inlineStr"/>
       <c r="I10" s="5" t="inlineStr"/>
       <c r="J10" s="5" t="inlineStr"/>
@@ -1200,7 +1221,10 @@
           <t>LNR_Insurance Fight PHX</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr"/>
+      <c r="G11" s="5">
+        <f>HYPERLINK("https://drive.google.com/file/d/1SQt6nyT4dFYs1biFWef3CaWheal-Crgq/view","▶ Watch")</f>
+        <v/>
+      </c>
       <c r="H11" s="5" t="inlineStr"/>
       <c r="I11" s="5" t="inlineStr"/>
       <c r="J11" s="5" t="inlineStr">
@@ -1349,7 +1373,10 @@
           <t>LNR_Eye Chart 26</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr"/>
+      <c r="G13" s="5">
+        <f>HYPERLINK("https://drive.google.com/file/d/1XDI7ApFLLZnSBpfYWQUHRI39hVeQwmDS/view","▶ Watch")</f>
+        <v/>
+      </c>
       <c r="H13" s="5" t="inlineStr"/>
       <c r="I13" s="5" t="inlineStr"/>
       <c r="J13" s="5" t="inlineStr"/>
@@ -1733,7 +1760,7 @@
         </is>
       </c>
       <c r="G18" s="5">
-        <f>HYPERLINK("https://wdvcseovujheftpzcoer.supabase.co/storage/v1/object/public/creative/PHXLR2615027T.mp4","▶ Watch")</f>
+        <f>HYPERLINK("https://drive.google.com/file/d/1PSBmU2B97zLJHBJl_WPK3wJxzjy2UcM0/view","▶ Watch")</f>
         <v/>
       </c>
       <c r="H18" s="5" t="inlineStr"/>

</xml_diff>